<commit_message>
logs 3 revery marketname lower'
</commit_message>
<xml_diff>
--- a/GII.xlsx
+++ b/GII.xlsx
@@ -544,23 +544,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Airsoft Guns Market Size, Share, and Growth Analysis, By Product Type (Handguns, Rifles), By Mechanism (Spring powered, Electric powered), By Price Range, By Distribution Channel, By Region - Industry Forecast 2025-2032</t>
+          <t>Power Tools Market Size, Share, and Growth Analysis, By Tool Type (Drilling And Fastening Tools, Demolition Tools), By Mode Of Operation (Electric, Pneumatic), By Application, By Region - Industry Forecast 2025-2032</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SQMIG25E2160</t>
+          <t>SQMIG20D2077</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.skyquestt.com/report/airsoft-guns-market%C2%A0</t>
+          <t>https://www.skyquestt.com/report/power-tools-market</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>193</t>
+          <t>157</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -581,17 +581,17 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Airsoft Guns Market size was valued at USD 2.1 billion in 2023 and is poised to grow from USD 2.27 billion in 2024 to USD 4.27 billion by 2032, growing at a CAGR of 8.2% during the forecast period (2025-2032).
-The airsoft guns market is experiencing robust growth, propelled by the rising popularity of recreational shooting and tactical sports. As more consumers engage in airsoft gaming events and competitive leagues, demand for high-quality, realistic airsoft guns is escalating. The market, segmented into electric, gas, and spring-powered models, favors electric airsoft guns (AEGs) for their rapid-fire capability and versatility. Innovations like 3D printing and gas blowback systems are enhancing product realism and durability, attracting both enthusiasts and military training programs. Recent product launches, such as Tokyo Marui's M4A1R and KRYTAC's gas-powered KRISS Vector, exemplify this trend towards advanced, affordable offerings. Despite regulatory hurdles, the market is set for steady growth, driven by technological advancements and an expanding consumer base.
-Top-down and bottom-up approaches were used to estimate and validate the size of the airsoft guns market and to estimate the size of various other dependent submarkets. The research methodology used to estimate the market size includes the following details: The key players in the market were identified through secondary research, and their market shares in the respective regions were determined through primary and secondary research. This entire procedure includes the study of the annual and financial reports of the top market players and extensive interviews for key insights from industry leaders such as CEOs, VPs, directors, and marketing executives. All percentage shares split, and breakdowns were determined using secondary sources and verified through Primary sources. All possible parameters that affect the markets covered in this research study have been accounted for, viewed in extensive detail, verified through primary research, and analyzed to get the final quantitative and qualitative data.
-airsoft guns Market Segments Analysis
-Global Airsoft Guns Market is segmented by Product Type, Mechanism, Price Range, Distribution Channel and region. Based on Product Type, the market is segmented into Handguns, Rifles, Shotgun and Muzzle loading. Based on Mechanism, the market is segmented into Spring powered, Electric powered and Gas powered. Based on Price Range, the market is segmented into Low (up to 100$), Mid (100$-200$) and High (above 300$). Based on Distribution Channel, the market is segmented into Online and Offline. Based on region, the market is segmented into North America, Europe, Asia Pacific, Latin America and Middle East &amp; Africa.
-Driver of the airsoft guns Market
-A significant driver of growth in the global airsoft guns market is the rising interest in airsoft sports, competitive tournaments, and military simulation activities. The surge in participation in organized airsoft leagues, coupled with the appeal of adventure tourism and tactical gaming communities, has led to an increased demand for high-performance airsoft guns, as well as essential accessories and realistic training equipment globally. This growing enthusiasm for airsoft as both a recreational activity and a competitive sport is propelling market expansion and fostering innovation in product offerings to meet the needs of passionate players.
-Restraints in the airsoft guns Market
-The airsoft guns market faces several constraints that hinder its growth, primarily due to stringent government regulations and legal limitations imposed in numerous countries. Many areas necessitate licensing, impose import bans, and categorize airsoft guns alongside firearms, creating obstacles for potential buyers. Additionally, concerns regarding public safety, potential weapon misuse, and the realistic appearance of these guns further exacerbate the regulatory challenges. These factors not only discourage consumers from making purchases but also impede the overall expansion of the global airsoft market, creating a complex landscape for manufacturers and retailers alike.
-Market Trends of the airsoft guns Market
-The airsoft guns market is witnessing a notable upward trend fueled by the burgeoning popularity of competitive airsoft sports and MilSim events. This increase in organized tournaments is prompting enthusiasts globally to invest in high-performance, realistic airsoft guns, enhancing their tactical gameplay experience. Additionally, the impact of social media and the integration of e-sports elements into airsoft competitions are broadening the appeal, successfully engaging a younger demographic. As brands innovate and cater to evolving consumer preferences, the market is set to expand further, establishing airsoft not just as a hobby but as a vibrant community-driven sport.</t>
+          <t>Power Tools Market size was valued at USD 37.5 billion in 2023 and is poised to grow from USD 39.68 billion in 2024 to USD 62.29 billion by 2032, growing at a CAGR of 5.8% during the forecast period (2025-2032).
+The power tools market is currently experiencing significant double-digit growth fueled by various factors in both developed and emerging economies. Notably, the rise in public infrastructure projects in markets like Brazil, Russia, India, China, South Africa, and Gulf Cooperation Council (GCC) countries is a key driver. With rapid population growth, nations like China and India are investing heavily in construction, leading to an increased demand for power tools across building, manufacturing, and maintenance sectors. Additionally, pandemic-induced behavioral shifts have spurred consumer interest in DIY projects, boosting sales of tools for home renovations. Looking ahead, anticipated investments in electric vehicle (EV) infrastructure, including 200 new gigafactories by 2030, will significantly elevate the requirement for power tools in this sector.
+Top-down and bottom-up approaches were used to estimate and validate the size of the Power Tools Market size was valued at USD 37.5 billion in 2023 and is poised to grow from USD 39.68 billion in 2024 to USD 62.29 billion by 2032, growing at a CAGR of 5.8% during the forecast period (2025-2032). market and to estimate the size of various other dependent submarkets. The research methodology used to estimate the market size includes the following details: The key players in the market were identified through secondary research, and their market shares in the respective regions were determined through primary and secondary research. This entire procedure includes the study of the annual and financial reports of the top market players and extensive interviews for key insights from industry leaders such as CEOs, VPs, directors, and marketing executives. All percentage shares split, and breakdowns were determined using secondary sources and verified through Primary sources. All possible parameters that affect the markets covered in this research study have been accounted for, viewed in extensive detail, verified through primary research, and analyzed to get the final quantitative and qualitative data.
+Power Tools Market size was valued at USD 37.5 billion in 2023 and is poised to grow from USD 39.68 billion in 2024 to USD 62.29 billion by 2032, growing at a CAGR of 5.8% during the forecast period (2025-2032). Market Segments Analysis
+Global Power Tools Market is segmented by Tool Type, Mode Of Operation, Application and region. Based on Tool Type, the market is segmented into Drilling And Fastening Tools, Demolition Tools, Sawing And Cutting Tools, Material Removal Tools, Routing Tools and Other Tools. Based on Mode Of Operation, the market is segmented into Electric, Pneumatic and Hydraulic. Based on Application, the market is segmented into Industrial/Professional and Residential/DIY. Based on region, the market is segmented into North America, Europe, Asia Pacific, Latin America and Middle East &amp; Africa.
+Driver of the Power Tools Market size was valued at USD 37.5 billion in 2023 and is poised to grow from USD 39.68 billion in 2024 to USD 62.29 billion by 2032, growing at a CAGR of 5.8% during the forecast period (2025-2032). Market
+One of the key market drivers for the global power tools market is the increasing demand for efficient and time-saving construction and manufacturing solutions. As urbanization and infrastructure development accelerate worldwide, there is a growing need for advanced power tools that enhance productivity and precision. The rise of DIY culture, particularly among millennials and homeowners seeking to undertake renovations and home improvements, further fuels this demand. Additionally, technological advancements in battery-powered and cordless tools are driving innovation and attracting both professional and amateur users, thus contributing to the market's robust growth forecasted from 2024 to 2032.
+Restraints in the Power Tools Market size was valued at USD 37.5 billion in 2023 and is poised to grow from USD 39.68 billion in 2024 to USD 62.29 billion by 2032, growing at a CAGR of 5.8% during the forecast period (2025-2032). Market
+The Power Tools Market is currently navigating several restraints that could hinder its growth. One significant challenge is the volatility in raw material prices, largely affecting the production of power tools, including power generators. Developed nations such as the United States, the United Kingdom, Japan, China, and India are projected to drive demand; however, fluctuating costs and economic instability pose risks. Many power tools are manufactured using steel, metals, and aluminum, materials that are often not locally sourced, resulting in price variations impacted by exchange rate fluctuations. These rising raw material costs consequently limit the overall growth potential of the market.
+Market Trends of the Power Tools Market size was valued at USD 37.5 billion in 2023 and is poised to grow from USD 39.68 billion in 2024 to USD 62.29 billion by 2032, growing at a CAGR of 5.8% during the forecast period (2025-2032). Market
+The Power Tools Market is experiencing a significant shift as it evolves towards sustainable and versatile solutions, with a market size valued at USD 37.5 billion in 2023, projected to grow to USD 62.29 billion by 2032, reflecting a robust CAGR of 5.8% from 2025 onwards. Leading companies like Atlas Copco AB and Robert Bosch Tool Corporation are at the forefront, introducing green energy technologies and multi-use cordless tools that cater to consumer preferences for lightweight, portable, and highly accurate devices. This demand for high-quality, efficient products drives innovation, positioning disruptive players to capitalize on the evolving landscape of the power tools industry.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -631,53 +631,66 @@
 o Macro-Economic Indicators
 o Value Chain Analysis
 o Pricing Analysis
-o Customer &amp; Buying Criteria Analysis
-• Global Airsoft Guns Market Size by Product Type &amp; CAGR (2025-2032)
+o Regulatory Analysis
+o Technology Analysis
+• Global Power Tools Market Size by Tool Type &amp; CAGR (2025-2032)
 o Market Overview
-o Handguns
-o Rifles
-o Shotgun
-o Muzzle loading
-• Global Airsoft Guns Market Size by Mechanism &amp; CAGR (2025-2032)
+o Drilling And Fastening Tools
+ Drills
+ Impact Drivers
+ Impact Wrenches
+ Screwdrivers And Nutrunners
+o Demolition Tools
+o Sawing And Cutting Tools
+ Jigsaws
+ Reciprocating Saws
+ Circular Saws
+ Band Saws
+ Shears &amp; Nibblers
+o Material Removal Tools
+ Sanders/Polishers/Buffers
+ Air Scalers
+ Grinders
+o Routing Tools
+o Other Tools
+• Global Power Tools Market Size by Mode Of Operation &amp; CAGR (2025-2032)
 o Market Overview
-o Spring powered
-o Electric powered
-o Gas powered
-• Global Airsoft Guns Market Size by Price Range &amp; CAGR (2025-2032)
+o Electric
+ Corded Tools
+ Cordless Tools
+o Pneumatic
+o Hydraulic
+• Global Power Tools Market Size by Application &amp; CAGR (2025-2032)
 o Market Overview
-o Low (up to 100$)
-o Mid (100$-200$)
-o High (above 300$)
-• Global Airsoft Guns Market Size by Distribution Channel &amp; CAGR (2025-2032)
-o Market Overview
-o Online
- E-commerce websites
- Company websites
-o Offline
- Hypermarket/supermarket
- Departmental stores
- Others
-• Global Airsoft Guns Market Size &amp; CAGR (2025-2032)
-o North America (Product Type, Mechanism, Price Range, Distribution Channel)
+o Industrial/Professional
+ Construction
+ Automotive
+ Aerospace
+ Energy
+ Shipbuilding
+ Other Industries
+o Residential/DIY
+• Global Power Tools Market Size &amp; CAGR (2025-2032)
+o North America (Tool Type, Mode Of Operation, Application)
  US
  Canada
-o Europe (Product Type, Mechanism, Price Range, Distribution Channel)
+o Europe (Tool Type, Mode Of Operation, Application)
  Germany
  Spain
  France
  UK
  Italy
  Rest of Europe
-o Asia Pacific (Product Type, Mechanism, Price Range, Distribution Channel)
+o Asia Pacific (Tool Type, Mode Of Operation, Application)
  China
  India
  Japan
  South Korea
  Rest of Asia-Pacific
-o Latin America (Product Type, Mechanism, Price Range, Distribution Channel)
+o Latin America (Tool Type, Mode Of Operation, Application)
  Brazil
  Rest of Latin America
-o Middle East &amp; Africa (Product Type, Mechanism, Price Range, Distribution Channel)
+o Middle East &amp; Africa (Tool Type, Mode Of Operation, Application)
  GCC Countries
  South Africa
  Rest of Middle East &amp; Africa
@@ -693,102 +706,87 @@
  Company's Segmental Share Analysis
  Revenue Y-O-Y Comparison (2022-2024)
 • Key Company Profiles
-o Tokyo Marui Co. Ltd. (Japan)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o G&amp;G Armament Taiwan Ltd. (Taiwan)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o Umarex GmbH &amp; Co. KG (Germany)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o ICS Airsoft Inc. (Taiwan)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o Lancer Tactical Inc. (USA)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o Colt's Manufacturing Company LLC (USA)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o Crosman Corporation (USA)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o Valken Inc. (USA)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o A&amp;K Airsoft Limited (China)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o HFC/Ballistic Breakthru Gunnery Corporation (Taiwan)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o Systema Professional Training Weapon (PTW) (Japan)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o KWA Performance Industries Inc. (USA)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o Classic Army (Hong Kong)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o VFC (Vega Force Company) (Taiwan)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o WE Airsoft (Taiwan)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o King Arms (Hong Kong)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o CYMA (China)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o Arcturus (Taiwan)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o ASG (ActionSportGames) (Denmark)
- Company Overview
- Business Segment Overview
- Financial Updates
- Key Developments
-o LCT Airsoft (Taiwan)
+o Robert Bosch GmbH (Germany)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Techtronic Industries Co. Ltd. (TTI) (Hong Kong)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Makita Corporation (Japan)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Hilti Corporation (Liechtenstein)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Atlas Copco AB (Sweden)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Snap-on Incorporated (US)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Emerson Electric Co. (US)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Chervon (China) Trading Co. Ltd. (China)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o TTI (Techtronic Industries) Power Tools (China)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Danaher Corporation (US)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Ingersoll Rand plc (Ireland)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o FEIN Power Tools Inc. (Germany)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Panasonic Corporation (Japan)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o KYOCERA Corporation (Japan)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Yamabiko Corporation (Japan)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Ken Holding Co., Ltd (China)
+ Company Overview
+ Business Segment Overview
+ Financial Updates
+ Key Developments
+o Dynabrade Inc. (US)
  Company Overview
  Business Segment Overview
  Financial Updates
@@ -800,7 +798,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -824,51 +822,48 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>◦ Tokyo Marui Co. Ltd. (Japan)
-◦ G&amp;G Armament Taiwan Ltd. (Taiwan)
-◦ Umarex GmbH &amp; Co. KG (Germany)
-◦ ICS Airsoft Inc. (Taiwan)
-◦ Lancer Tactical Inc. (USA)
-◦ Colt's Manufacturing Company LLC (USA)
-◦ Crosman Corporation (USA)
-◦ Valken Inc. (USA)
-◦ A&amp;K Airsoft Limited (China)
-◦ HFC/Ballistic Breakthru Gunnery Corporation (Taiwan)
-◦ Systema Professional Training Weapon (PTW) (Japan)
-◦ KWA Performance Industries Inc. (USA)
-◦ Classic Army (Hong Kong)
-◦ VFC (Vega Force Company) (Taiwan)
-◦ WE Airsoft (Taiwan)
-◦ King Arms (Hong Kong)
-◦ CYMA (China)
-◦ Arcturus (Taiwan)
-◦ ASG (ActionSportGames) (Denmark)
-◦ LCT Airsoft (Taiwan)</t>
+          <t>◦ Robert Bosch GmbH (Germany)
+◦ Techtronic Industries Co. Ltd. (TTI) (Hong Kong)
+◦ Makita Corporation (Japan)
+◦ Hilti Corporation (Liechtenstein)
+◦ Atlas Copco AB (Sweden)
+◦ Snap-on Incorporated (US)
+◦ Emerson Electric Co. (US)
+◦ Chervon (China) Trading Co. Ltd. (China)
+◦ TTI (Techtronic Industries) Power Tools (China)
+◦ Danaher Corporation (US)
+◦ Ingersoll Rand plc (Ireland)
+◦ FEIN Power Tools Inc. (Germany)
+◦ Panasonic Corporation (Japan)
+◦ KYOCERA Corporation (Japan)
+◦ Yamabiko Corporation (Japan)
+◦ Ken Holding Co., Ltd (China)
+◦ Dynabrade Inc. (US)</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>By Product Type (Handguns, Rifles, Shotgun, Muzzle Loading), By Mechanism (Spring Powered, Electric Powered, Gas Powered), By Price Range (Low (up to 100$), Mid (100$-200$), High (above 300$)), By Distribution Channel (Online (E-commerce websites, Company websites), Offline (Hypermarket/supermarket, Departmental stores, Others))</t>
+          <t>By Tool Type (Drilling And Fastening Tools (Drills, Impact Drivers, Impact Wrenches, Screwdrivers And Nutrunners), Demolition Tools, Sawing And Cutting Tools (Jigsaws, Reciprocating Saws, Circular Saws, Band Saws, Shears &amp; Nibblers), Material Removal Tools, Routing Tools, Other Tools), By Mode Of Operation (Electric (Corded Tools, Cordless Tools), Pneumatic, Hydraulic), By Application (Industrial/Professional (Construction, Automotive, Aerospace, Energy, Shipbuilding, Other Industries), Residential/DIY)</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>37.5</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>39.68</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>4.27</t>
+          <t>62.29</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>5.8%</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">

</xml_diff>